<commit_message>
Finished stores domain and added vendor domain
</commit_message>
<xml_diff>
--- a/WorkBot/main/data/orders/Albert's Organics/combined_orders_Albert's Organics.xlsx
+++ b/WorkBot/main/data/orders/Albert's Organics/combined_orders_Albert's Organics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andrew\Desktop\Andrew\Projects\IthacaBakery\RandomStuff\WorkBot\main\data\orders\Albert's Organics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6584A36-7884-40C0-85B9-DCF9056390BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FE66894-7B1A-4509-81C1-7FE6223C9108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5040" yWindow="3210" windowWidth="16200" windowHeight="9360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Item Name</t>
   </si>
@@ -45,12 +45,15 @@
     <t>Downtown</t>
   </si>
   <si>
-    <t>Easthill</t>
+    <t>Triphammer</t>
   </si>
   <si>
     <t>Chow Maine - Kale Pesto Pasta</t>
   </si>
   <si>
+    <t>Chow Maine - Kale Tofu Salad</t>
+  </si>
+  <si>
     <t>Chow Maine - Sesame Noodle Salad</t>
   </si>
   <si>
@@ -60,12 +63,15 @@
     <t>Chow Maine - Thai Noodle Salad</t>
   </si>
   <si>
-    <t>Harney &amp; Sons - Green with Coconut</t>
+    <t>Natalie's - Honey Tangerine</t>
   </si>
   <si>
     <t>Niman Ranch Snack Pk - HotSporessata, Olives, Prov</t>
   </si>
   <si>
+    <t>Niman Ranch Snack Pk - Pepperoni, Choc, Prov</t>
+  </si>
+  <si>
     <t>Niman Ranch Snack Pk - Salame, Taralli, Prov</t>
   </si>
   <si>
@@ -73,6 +79,9 @@
   </si>
   <si>
     <t>Painterland Sisters - Icelandic Skyr Strawberry</t>
+  </si>
+  <si>
+    <t>Painterland Sisters - Meadowberry Yogurt</t>
   </si>
   <si>
     <t>Painterland Sisters - Savanah Peach Yogurt</t>
@@ -102,7 +111,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -110,13 +119,154 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="dotted">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="dotted">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="dotted">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="dotted">
+        <color auto="1"/>
+      </top>
+      <bottom style="dotted">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="dotted">
+        <color auto="1"/>
+      </top>
+      <bottom style="dotted">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="dotted">
+        <color auto="1"/>
+      </top>
+      <bottom style="dotted">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="dotted">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="dotted">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="dotted">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -421,140 +571,214 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="13.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="47.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="11.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="7">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="7">
+        <v>1</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1">
+      <c r="B5" s="7">
+        <v>1</v>
+      </c>
+      <c r="C5" s="7">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="1">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1">
+      <c r="B6" s="7">
+        <v>1</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1">
-        <v>1</v>
-      </c>
+      <c r="B7" s="7">
+        <v>1</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="8"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="1">
-        <v>1</v>
-      </c>
+      <c r="B8" s="7">
+        <v>1</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="8"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="1">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1">
-        <v>1</v>
-      </c>
-      <c r="D9" s="1">
-        <v>1</v>
-      </c>
+      <c r="B9" s="7">
+        <v>1</v>
+      </c>
+      <c r="C9" s="7">
+        <v>1</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="1">
-        <v>1</v>
-      </c>
-      <c r="D10" s="1">
-        <v>1</v>
-      </c>
-      <c r="E10" s="1">
-        <v>1</v>
-      </c>
+      <c r="B10" s="7">
+        <v>1</v>
+      </c>
+      <c r="C10" s="7">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="8"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="7">
+        <v>1</v>
+      </c>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="A12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="1">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7">
+        <v>1</v>
+      </c>
+      <c r="E12" s="8"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7">
+        <v>1</v>
+      </c>
+      <c r="E13" s="8"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="7">
+        <v>1</v>
+      </c>
+      <c r="C14" s="7">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7"/>
+      <c r="E14" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10">
+        <v>1</v>
+      </c>
+      <c r="D15" s="10">
+        <v>1</v>
+      </c>
+      <c r="E15" s="11">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>